<commit_message>
test/update supplier execution test cases.
</commit_message>
<xml_diff>
--- a/TestCases_Docs/Supplier_Tcs.xlsx
+++ b/TestCases_Docs/Supplier_Tcs.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\iti\QA\New folder\Clothing-Web-Portal\TestCases_Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA29B224-5C2F-4637-8D30-08A373A75E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9DD12DA-2BE0-4335-828D-629776E4B400}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11520" windowHeight="12360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier_Tcs" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="138">
   <si>
     <t>TesTCASE ID</t>
   </si>
@@ -398,9 +398,6 @@
   </si>
   <si>
     <t>Pass</t>
-  </si>
-  <si>
-    <t>Fail</t>
   </si>
   <si>
     <t>Executed by</t>
@@ -1005,7 +1002,7 @@
         <v>50</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>20</v>
@@ -1062,7 +1059,7 @@
         <v>50</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>20</v>
@@ -1119,7 +1116,7 @@
         <v>53</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>20</v>
@@ -1176,7 +1173,7 @@
         <v>30</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>20</v>
@@ -1233,7 +1230,7 @@
         <v>56</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>20</v>
@@ -1288,7 +1285,7 @@
         <v>41</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K7" s="4" t="s">
         <v>20</v>
@@ -1345,7 +1342,7 @@
         <v>62</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K8" s="4" t="s">
         <v>20</v>
@@ -1402,7 +1399,7 @@
         <v>68</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>20</v>
@@ -1459,7 +1456,7 @@
         <v>81</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>20</v>
@@ -1516,7 +1513,7 @@
         <v>66</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>20</v>
@@ -1573,7 +1570,7 @@
         <v>74</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>20</v>
@@ -1630,7 +1627,7 @@
         <v>90</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>20</v>
@@ -1687,7 +1684,7 @@
         <v>96</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>20</v>
@@ -1744,7 +1741,7 @@
         <v>100</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>20</v>
@@ -1801,7 +1798,7 @@
         <v>107</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K16" s="6" t="s">
         <v>20</v>
@@ -29947,7 +29944,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>4</v>
@@ -29965,7 +29962,7 @@
         <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>114</v>
@@ -29980,10 +29977,10 @@
         <v>12</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" s="1" t="s">
         <v>117</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="O1" s="1" t="s">
         <v>3</v>
@@ -30012,13 +30009,13 @@
         <v>50</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>21</v>
@@ -30027,7 +30024,7 @@
         <v>22</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>23</v>
@@ -30053,19 +30050,19 @@
         <v>20</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>50</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="I3" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K3" s="4" t="s">
         <v>21</v>
@@ -30074,7 +30071,7 @@
         <v>22</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N3" s="4" t="s">
         <v>23</v>
@@ -30106,13 +30103,13 @@
         <v>53</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K4" s="4" t="s">
         <v>21</v>
@@ -30121,7 +30118,7 @@
         <v>22</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N4" s="4" t="s">
         <v>23</v>
@@ -30153,13 +30150,13 @@
         <v>30</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K5" s="4" t="s">
         <v>21</v>
@@ -30168,7 +30165,7 @@
         <v>22</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N5" s="4" t="s">
         <v>23</v>
@@ -30200,13 +30197,13 @@
         <v>56</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K6" s="4" t="s">
         <v>36</v>
@@ -30215,7 +30212,7 @@
         <v>22</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N6" s="4" t="s">
         <v>23</v>
@@ -30258,7 +30255,7 @@
         <v>22</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N7" s="4" t="s">
         <v>23</v>
@@ -30303,7 +30300,7 @@
         <v>22</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N8" s="4" t="s">
         <v>23</v>
@@ -30335,13 +30332,13 @@
         <v>68</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I9" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K9" s="4" t="s">
         <v>45</v>
@@ -30350,7 +30347,7 @@
         <v>22</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N9" s="4" t="s">
         <v>23</v>
@@ -30382,13 +30379,13 @@
         <v>81</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I10" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K10" s="4" t="s">
         <v>45</v>
@@ -30397,7 +30394,7 @@
         <v>22</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N10" s="4" t="s">
         <v>23</v>
@@ -30429,13 +30426,13 @@
         <v>66</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="I11" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K11" s="4" t="s">
         <v>45</v>
@@ -30444,7 +30441,7 @@
         <v>22</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N11" s="4" t="s">
         <v>23</v>
@@ -30476,13 +30473,13 @@
         <v>74</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I12" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K12" s="4" t="s">
         <v>75</v>
@@ -30491,7 +30488,7 @@
         <v>22</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N12" s="4" t="s">
         <v>23</v>
@@ -30523,13 +30520,13 @@
         <v>90</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I13" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K13" s="4" t="s">
         <v>75</v>
@@ -30538,7 +30535,7 @@
         <v>22</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N13" s="4" t="s">
         <v>23</v>
@@ -30570,13 +30567,13 @@
         <v>96</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I14" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K14" s="4" t="s">
         <v>75</v>
@@ -30585,7 +30582,7 @@
         <v>22</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N14" s="4" t="s">
         <v>23</v>
@@ -30617,13 +30614,13 @@
         <v>100</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I15" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K15" s="4" t="s">
         <v>101</v>
@@ -30632,7 +30629,7 @@
         <v>22</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N15" s="4" t="s">
         <v>23</v>
@@ -30664,13 +30661,13 @@
         <v>107</v>
       </c>
       <c r="H16" s="28" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I16" s="4" t="s">
         <v>115</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K16" s="10" t="s">
         <v>108</v>
@@ -30679,7 +30676,7 @@
         <v>22</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N16" s="10" t="s">
         <v>23</v>

</xml_diff>